<commit_message>
dual portfolio done till summary
</commit_message>
<xml_diff>
--- a/electron/data/summary.xlsx
+++ b/electron/data/summary.xlsx
@@ -475,16 +475,16 @@
         <v>178.81973275531917</v>
       </c>
       <c r="I2">
-        <v>217.87</v>
+        <v>219.49</v>
       </c>
       <c r="J2">
-        <v>5.55</v>
+        <v>-2.19</v>
       </c>
       <c r="K2" t="str">
-        <v>(2.61%)</v>
+        <v>(-0.99%)</v>
       </c>
       <c r="L2">
-        <v>21.837784143271097</v>
+        <v>22.74372443019495</v>
       </c>
       <c r="M2">
         <v>10.42753148506382</v>
@@ -522,16 +522,16 @@
         <v>222.71513564555553</v>
       </c>
       <c r="I3">
-        <v>404.15</v>
+        <v>437</v>
       </c>
       <c r="J3">
-        <v>3.86</v>
+        <v>1.02</v>
       </c>
       <c r="K3" t="str">
-        <v>(0.96%)</v>
+        <v>(0.23%)</v>
       </c>
       <c r="L3">
-        <v>81.46499061617105</v>
+        <v>96.21477396824632</v>
       </c>
       <c r="M3">
         <v>36.84314366452076</v>
@@ -569,16 +569,16 @@
         <v>14.116166666666667</v>
       </c>
       <c r="I4">
-        <v>16.9</v>
+        <v>17.45</v>
       </c>
       <c r="J4">
-        <v>0.14</v>
+        <v>-0.11</v>
       </c>
       <c r="K4" t="str">
-        <v>(0.84%)</v>
+        <v>(-0.63%)</v>
       </c>
       <c r="L4">
-        <v>19.72088739860915</v>
+        <v>23.617129296197028</v>
       </c>
       <c r="M4">
         <v>8.756992788986127</v>
@@ -601,7 +601,7 @@
         <v>Mari Energies Limited</v>
       </c>
       <c r="D5" t="str">
-        <v>XD</v>
+        <v/>
       </c>
       <c r="E5" t="str">
         <v>OIL &amp; GAS EXPLORATION COMPANIES</v>
@@ -616,16 +616,16 @@
         <v>601.8757826767677</v>
       </c>
       <c r="I5">
-        <v>706.4</v>
+        <v>760.9</v>
       </c>
       <c r="J5">
-        <v>18.78</v>
+        <v>19.86</v>
       </c>
       <c r="K5" t="str">
-        <v>(2.73%)</v>
+        <v>(2.68%)</v>
       </c>
       <c r="L5">
-        <v>17.36641020151597</v>
+        <v>26.42143477114029</v>
       </c>
       <c r="M5">
         <v>24.64274139522381</v>
@@ -663,16 +663,16 @@
         <v>25.82693091549296</v>
       </c>
       <c r="I6">
-        <v>32.03</v>
+        <v>32</v>
       </c>
       <c r="J6">
-        <v>-0.02</v>
+        <v>-0.09</v>
       </c>
       <c r="K6" t="str">
-        <v>(-0.06%)</v>
+        <v>(-0.28%)</v>
       </c>
       <c r="L6">
-        <v>24.017832799428636</v>
+        <v>23.90167497913569</v>
       </c>
       <c r="M6">
         <v>7.583646926333468</v>
@@ -710,16 +710,16 @@
         <v>17.5295</v>
       </c>
       <c r="I7">
-        <v>20.63</v>
+        <v>21.1</v>
       </c>
       <c r="J7">
-        <v>0.05</v>
+        <v>-0.18</v>
       </c>
       <c r="K7" t="str">
-        <v>(0.24%)</v>
+        <v>(-0.85%)</v>
       </c>
       <c r="L7">
-        <v>17.6873270772127</v>
+        <v>20.36852163495823</v>
       </c>
       <c r="M7">
         <v>3.624820361867181</v>
@@ -757,16 +757,16 @@
         <v>371.33569240624996</v>
       </c>
       <c r="I8">
-        <v>464.62</v>
+        <v>472.99</v>
       </c>
       <c r="J8">
-        <v>-10.21</v>
+        <v>-2.9</v>
       </c>
       <c r="K8" t="str">
-        <v>(-2.15%)</v>
+        <v>(-0.61%)</v>
       </c>
       <c r="L8">
-        <v>25.121287692348954</v>
+        <v>27.375312869881046</v>
       </c>
       <c r="M8">
         <v>1.2285805563624501</v>
@@ -804,16 +804,16 @@
         <v>122.74421769642858</v>
       </c>
       <c r="I9">
-        <v>143.21</v>
+        <v>151.49</v>
       </c>
       <c r="J9">
-        <v>-0.81</v>
+        <v>0.24</v>
       </c>
       <c r="K9" t="str">
-        <v>(-0.56%)</v>
+        <v>(0.16%)</v>
       </c>
       <c r="L9">
-        <v>16.67352050276411</v>
+        <v>23.4192557849573</v>
       </c>
       <c r="M9">
         <v>3.5534158729596457</v>
@@ -851,16 +851,16 @@
         <v>836.69580625</v>
       </c>
       <c r="I10">
-        <v>926.95</v>
+        <v>900</v>
       </c>
       <c r="J10">
-        <v>5.29</v>
+        <v>-2.13</v>
       </c>
       <c r="K10" t="str">
-        <v>(0.57%)</v>
+        <v>(-0.24%)</v>
       </c>
       <c r="L10">
-        <v>10.786978143766692</v>
+        <v>7.5659747876261045</v>
       </c>
       <c r="M10">
         <v>1.3841225340980075</v>
@@ -869,7 +869,7 @@
         <v>0</v>
       </c>
       <c r="O10">
-        <v>40</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11">
@@ -898,13 +898,13 @@
         <v>1470.8712083333332</v>
       </c>
       <c r="I11" t="str">
-        <v>1,715.57</v>
+        <v>1,889.94</v>
       </c>
       <c r="J11">
-        <v>12.57</v>
+        <v>81.51</v>
       </c>
       <c r="K11" t="str">
-        <v>(0.74%)</v>
+        <v>(4.51%)</v>
       </c>
       <c r="M11">
         <v>1.8249159094044385</v>
@@ -942,16 +942,16 @@
         <v>260.4535</v>
       </c>
       <c r="I12">
-        <v>277.88</v>
+        <v>278.5</v>
       </c>
       <c r="J12">
-        <v>-4.98</v>
+        <v>1.27</v>
       </c>
       <c r="K12" t="str">
-        <v>(-1.76%)</v>
+        <v>(0.46%)</v>
       </c>
       <c r="L12">
-        <v>6.690829649054428</v>
+        <v>6.928875979781411</v>
       </c>
       <c r="M12">
         <v>0.10771524003760219</v>
@@ -989,16 +989,16 @@
         <v>54.09815</v>
       </c>
       <c r="I13">
-        <v>54.37</v>
+        <v>56.35</v>
       </c>
       <c r="J13">
-        <v>-0.03</v>
+        <v>-0.33</v>
       </c>
       <c r="K13" t="str">
-        <v>(-0.05%)</v>
+        <v>(-0.58%)</v>
       </c>
       <c r="L13">
-        <v>0.5025125628140715</v>
+        <v>4.162526814687757</v>
       </c>
       <c r="M13">
         <v>0.022373265142684617</v>

</xml_diff>